<commit_message>
fixed business days value format, added TB match process functions
</commit_message>
<xml_diff>
--- a/categories_index.xlsx
+++ b/categories_index.xlsx
@@ -434,22 +434,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>threshold</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>client</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>client_id</t>
         </is>
@@ -900,29 +900,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>threshold</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>client</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>client_id</t>
         </is>
@@ -1338,6 +1338,13 @@
       <c r="A60" t="inlineStr">
         <is>
           <t>6703 Payroll Taxes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>62000 Business Licenses and Taxes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added green tint to all passed recon TB matches, added env settable theshold for recon, added double colon fix
</commit_message>
<xml_diff>
--- a/categories_index.xlsx
+++ b/categories_index.xlsx
@@ -4,22 +4,96 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" tabRatio="600" autoFilterDateGrouping="true"/>
   </bookViews>
   <sheets>
-    <sheet name="wages" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="pr_taxes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="pr_fees" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="subscriptions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="utilities" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="wages" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="pr_taxes" sheetId="2" r:id="rId2" state="visible"/>
+    <sheet name="pr_fees" sheetId="3" r:id="rId3" state="visible"/>
+    <sheet name="subscriptions" sheetId="4" r:id="rId4" state="visible"/>
+    <sheet name="utilities" sheetId="5" r:id="rId5" state="visible"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>5150 Direct Labor - Bonus</t>
+  </si>
+  <si>
+    <t>5150 Direct Labor - Bonuses</t>
+  </si>
+  <si>
+    <t>1-65520 Bonuses</t>
+  </si>
+  <si>
+    <t>2401 Accrued Bonuses</t>
+  </si>
+  <si>
+    <t>3-65520 Bonuses</t>
+  </si>
+  <si>
+    <t>5023 DL - Bonus</t>
+  </si>
+  <si>
+    <t>60005 Bonus</t>
+  </si>
+  <si>
+    <t>60006 Bonus</t>
+  </si>
+  <si>
+    <t>6004 Employee Bonus</t>
+  </si>
+  <si>
+    <t>60040 Bonus</t>
+  </si>
+  <si>
+    <t>60050 Bonus</t>
+  </si>
+  <si>
+    <t>6009 Bonus</t>
+  </si>
+  <si>
+    <t>6023 Employee Bonus</t>
+  </si>
+  <si>
+    <t>6024 Employee PR - Bonuses</t>
+  </si>
+  <si>
+    <t>6025 Employee Bonuses</t>
+  </si>
+  <si>
+    <t>6111 Employee PR - Bonus</t>
+  </si>
+  <si>
+    <t>6359 Margin Bonus</t>
+  </si>
+  <si>
+    <t>6361 Bonus &amp; Incentives</t>
+  </si>
+  <si>
+    <t>6404 Employee Bonus</t>
+  </si>
+  <si>
+    <t>64500 Bonus</t>
+  </si>
+  <si>
+    <t>6555 Bonus</t>
+  </si>
+  <si>
+    <t>6709 Bonus</t>
+  </si>
+  <si>
+    <t>60002 Officer Bonus</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="0"/>
   <fonts count="2">
     <font>
@@ -60,13 +134,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="false" pivotButton="false"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" quotePrefix="false" pivotButton="false"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="false"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -139,7 +213,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -422,15 +496,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col customWidth="true" max="1" min="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -887,6 +961,121 @@
         <is>
           <t>6701 Salaries &amp; Wages</t>
         </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed false green tint, added 15 percent value throughout categories_index and added no threshold found warning for matched rows with no threshold
</commit_message>
<xml_diff>
--- a/categories_index.xlsx
+++ b/categories_index.xlsx
@@ -535,6 +535,9 @@
           <t>1-22800 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B2">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -542,6 +545,9 @@
           <t>1-65530 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B3">
+        <v>15</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -549,6 +555,9 @@
           <t>1-65540 Tech Salaries</t>
         </is>
       </c>
+      <c r="B4">
+        <v>15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -556,6 +565,9 @@
           <t>21102 Contractor Wages P...</t>
         </is>
       </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -563,6 +575,9 @@
           <t>2200 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -570,6 +585,9 @@
           <t>2200 Wages Payable</t>
         </is>
       </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -577,6 +595,9 @@
           <t>22000 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -584,6 +605,9 @@
           <t>22000 Wages Payable</t>
         </is>
       </c>
+      <c r="B9">
+        <v>15</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -591,6 +615,9 @@
           <t>2201 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -598,6 +625,9 @@
           <t>22010 Salaries &amp; Wages Payable</t>
         </is>
       </c>
+      <c r="B11">
+        <v>15</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -605,6 +635,9 @@
           <t>2210 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -612,6 +645,9 @@
           <t>2215 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B13">
+        <v>15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -619,6 +655,9 @@
           <t>2310 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B14">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -626,6 +665,9 @@
           <t>2400 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B15">
+        <v>15</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -633,6 +675,9 @@
           <t>24000 Payroll Liabilities</t>
         </is>
       </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -640,6 +685,9 @@
           <t>3-65530 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -647,6 +695,9 @@
           <t>4-65530 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B18">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -654,6 +705,9 @@
           <t>5001 Direct Labor - Wages</t>
         </is>
       </c>
+      <c r="B19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -661,6 +715,9 @@
           <t>5001 Direct Labor Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B20">
+        <v>15</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -668,6 +725,9 @@
           <t>5001 Direct Wages</t>
         </is>
       </c>
+      <c r="B21">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -675,6 +735,9 @@
           <t>50063 Fulfillment Center Wages</t>
         </is>
       </c>
+      <c r="B22">
+        <v>15</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -682,6 +745,9 @@
           <t>5021 DL - EE Wages</t>
         </is>
       </c>
+      <c r="B23">
+        <v>15</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -689,6 +755,9 @@
           <t>5021 Employee PR - DL Wages</t>
         </is>
       </c>
+      <c r="B24">
+        <v>15</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -696,6 +765,9 @@
           <t>5100 Direct Salaries &amp; Benefits</t>
         </is>
       </c>
+      <c r="B25">
+        <v>15</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -703,6 +775,9 @@
           <t>5101 Direct Labor PR - Wages</t>
         </is>
       </c>
+      <c r="B26">
+        <v>15</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -710,6 +785,9 @@
           <t>5101 Direct Wages</t>
         </is>
       </c>
+      <c r="B27">
+        <v>15</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -717,6 +795,9 @@
           <t>5110 Direct Labor - Wages</t>
         </is>
       </c>
+      <c r="B28">
+        <v>15</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -724,6 +805,9 @@
           <t>51110-000 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B29">
+        <v>15</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -731,6 +815,9 @@
           <t>5130 Direct Labor - OT</t>
         </is>
       </c>
+      <c r="B30">
+        <v>15</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -738,6 +825,9 @@
           <t>5140 Direct Labor - PTO</t>
         </is>
       </c>
+      <c r="B31">
+        <v>15</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -745,6 +835,9 @@
           <t>5185 Direct Labor - Other Benefits</t>
         </is>
       </c>
+      <c r="B32">
+        <v>15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -752,6 +845,9 @@
           <t>52101-000 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B33">
+        <v>15</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -759,6 +855,9 @@
           <t>5221 The TREAD Agency - DL Wages</t>
         </is>
       </c>
+      <c r="B34">
+        <v>15</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -766,6 +865,9 @@
           <t>53101-000 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -773,6 +875,9 @@
           <t>5503 Sales - Salary</t>
         </is>
       </c>
+      <c r="B36">
+        <v>15</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -780,6 +885,9 @@
           <t>60001 Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B37">
+        <v>15</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -787,6 +895,9 @@
           <t>60002 Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B38">
+        <v>15</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -794,6 +905,9 @@
           <t>6001 Wages</t>
         </is>
       </c>
+      <c r="B39">
+        <v>15</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -801,6 +915,9 @@
           <t>60010 Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B40">
+        <v>15</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -808,6 +925,9 @@
           <t>60011-000 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B41">
+        <v>15</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -815,6 +935,9 @@
           <t>6002 Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B42">
+        <v>15</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -822,6 +945,9 @@
           <t>60020 Wages</t>
         </is>
       </c>
+      <c r="B43">
+        <v>15</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -829,6 +955,9 @@
           <t>6003 Indirect Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B44">
+        <v>15</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -836,6 +965,9 @@
           <t>6021 Employee PR - Wages</t>
         </is>
       </c>
+      <c r="B45">
+        <v>15</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -843,6 +975,9 @@
           <t>6021 Employee Wages</t>
         </is>
       </c>
+      <c r="B46">
+        <v>15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -850,6 +985,9 @@
           <t>6022 Wages</t>
         </is>
       </c>
+      <c r="B47">
+        <v>15</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -857,6 +995,9 @@
           <t>6030 Wages</t>
         </is>
       </c>
+      <c r="B48">
+        <v>15</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -864,6 +1005,9 @@
           <t>6100 Indirect Salaries &amp; Benefits</t>
         </is>
       </c>
+      <c r="B49">
+        <v>15</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -871,6 +1015,9 @@
           <t>6101 Employee PR - Wages</t>
         </is>
       </c>
+      <c r="B50">
+        <v>15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -878,6 +1025,9 @@
           <t>6101.2 Wages - Social Media Ma...</t>
         </is>
       </c>
+      <c r="B51">
+        <v>15</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -885,6 +1035,9 @@
           <t>6101.3 Wages - Social Media Ad...</t>
         </is>
       </c>
+      <c r="B52">
+        <v>15</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -892,6 +1045,9 @@
           <t>6101.4 Wages - SEM</t>
         </is>
       </c>
+      <c r="B53">
+        <v>15</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -899,6 +1055,9 @@
           <t>6101.5 Wages - Sales</t>
         </is>
       </c>
+      <c r="B54">
+        <v>15</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -906,6 +1065,9 @@
           <t>6101.6 Wages - Video</t>
         </is>
       </c>
+      <c r="B55">
+        <v>15</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -913,6 +1075,9 @@
           <t>6110 Employee PR - Wages</t>
         </is>
       </c>
+      <c r="B56">
+        <v>15</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -920,6 +1085,9 @@
           <t>6356 Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B57">
+        <v>15</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -927,6 +1095,9 @@
           <t>6401 Employee Wages</t>
         </is>
       </c>
+      <c r="B58">
+        <v>15</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -934,6 +1105,9 @@
           <t>64100 Wages</t>
         </is>
       </c>
+      <c r="B59">
+        <v>15</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -941,6 +1115,9 @@
           <t>6451 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B60">
+        <v>15</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -948,6 +1125,9 @@
           <t>65101-000 Salaries and Wages</t>
         </is>
       </c>
+      <c r="B61">
+        <v>15</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -955,91 +1135,145 @@
           <t>6551 Salaries &amp; Wages</t>
         </is>
       </c>
+      <c r="B62">
+        <v>15</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
           <t>6701 Salaries &amp; Wages</t>
         </is>
+      </c>
+      <c r="B63">
+        <v>15</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
         <v>0</v>
       </c>
+      <c r="B64">
+        <v>15</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
         <v>1</v>
       </c>
+      <c r="B65">
+        <v>15</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
         <v>2</v>
       </c>
+      <c r="B66">
+        <v>15</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
         <v>3</v>
       </c>
+      <c r="B67">
+        <v>15</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
         <v>4</v>
       </c>
+      <c r="B68">
+        <v>15</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
         <v>5</v>
       </c>
+      <c r="B69">
+        <v>15</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
         <v>6</v>
       </c>
+      <c r="B70">
+        <v>15</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
         <v>7</v>
       </c>
+      <c r="B71">
+        <v>15</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
         <v>8</v>
       </c>
+      <c r="B72">
+        <v>15</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
         <v>9</v>
       </c>
+      <c r="B73">
+        <v>15</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
         <v>10</v>
       </c>
+      <c r="B74">
+        <v>15</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
         <v>11</v>
       </c>
+      <c r="B75">
+        <v>15</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
         <v>12</v>
       </c>
+      <c r="B76">
+        <v>15</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
         <v>13</v>
       </c>
+      <c r="B77">
+        <v>15</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
         <v>14</v>
       </c>
+      <c r="B78">
+        <v>15</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
+        <v>15</v>
+      </c>
+      <c r="B79">
         <v>15</v>
       </c>
     </row>
@@ -1047,35 +1281,56 @@
       <c r="A80" t="s">
         <v>16</v>
       </c>
+      <c r="B80">
+        <v>15</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
         <v>17</v>
       </c>
+      <c r="B81">
+        <v>15</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
         <v>18</v>
       </c>
+      <c r="B82">
+        <v>15</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
         <v>19</v>
       </c>
+      <c r="B83">
+        <v>15</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
         <v>20</v>
       </c>
+      <c r="B84">
+        <v>15</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
         <v>21</v>
       </c>
+      <c r="B85">
+        <v>15</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
         <v>22</v>
+      </c>
+      <c r="B86">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1084,15 +1339,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col customWidth="true" max="1" min="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1123,6 +1378,9 @@
           <t>1-65550 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B2">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1130,6 +1388,9 @@
           <t>2202 CA PIT / SDI</t>
         </is>
       </c>
+      <c r="B3">
+        <v>15</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1137,6 +1398,9 @@
           <t>2202 Federal Taxes (941/943/944)</t>
         </is>
       </c>
+      <c r="B4">
+        <v>15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1144,6 +1408,9 @@
           <t>2203 CA PIT / SDI</t>
         </is>
       </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1151,6 +1418,9 @@
           <t>2203 CA SUI / ETT</t>
         </is>
       </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1158,6 +1428,9 @@
           <t>2203 Federal Taxes (941/944)</t>
         </is>
       </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1165,6 +1438,9 @@
           <t>2203 Federal Unemployment (940)</t>
         </is>
       </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1172,6 +1448,9 @@
           <t>2204 CA SUI / ETT</t>
         </is>
       </c>
+      <c r="B9">
+        <v>15</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1179,6 +1458,9 @@
           <t>2204 Federal Taxes (941/943/944)</t>
         </is>
       </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1186,6 +1468,9 @@
           <t>2204 Federal Unemployment (940)</t>
         </is>
       </c>
+      <c r="B11">
+        <v>15</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1193,6 +1478,9 @@
           <t>2205 Federal Unemployment (940)</t>
         </is>
       </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1200,6 +1488,9 @@
           <t>2206 Federal Taxes (941/944)</t>
         </is>
       </c>
+      <c r="B13">
+        <v>15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1207,6 +1498,9 @@
           <t>2207 Federal Unemployment (940)</t>
         </is>
       </c>
+      <c r="B14">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1214,6 +1508,9 @@
           <t>2207 Payroll Tax Liabilities</t>
         </is>
       </c>
+      <c r="B15">
+        <v>15</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1221,6 +1518,9 @@
           <t>2220 Payroll taxes payable</t>
         </is>
       </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1228,6 +1528,9 @@
           <t>22200-003 Payroll tax paya...</t>
         </is>
       </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1235,6 +1538,9 @@
           <t>2311 CA PIT / SDI</t>
         </is>
       </c>
+      <c r="B18">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1242,6 +1548,9 @@
           <t>2312 CA SUI / ETT</t>
         </is>
       </c>
+      <c r="B19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1249,6 +1558,9 @@
           <t>2313 Federal Taxes (941/944)</t>
         </is>
       </c>
+      <c r="B20">
+        <v>15</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1256,6 +1568,9 @@
           <t>2315 Payroll Taxes Employee</t>
         </is>
       </c>
+      <c r="B21">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1263,6 +1578,9 @@
           <t>2401 CA PIT / SDI</t>
         </is>
       </c>
+      <c r="B22">
+        <v>15</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1270,6 +1588,9 @@
           <t>2402 ADP Payroll Tax Withheld</t>
         </is>
       </c>
+      <c r="B23">
+        <v>15</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1277,6 +1598,9 @@
           <t>2402 CA SUI / ETT</t>
         </is>
       </c>
+      <c r="B24">
+        <v>15</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1284,6 +1608,9 @@
           <t>2403 Federal Taxes (941/...</t>
         </is>
       </c>
+      <c r="B25">
+        <v>15</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1291,6 +1618,9 @@
           <t>24031 CA PIT / SDI</t>
         </is>
       </c>
+      <c r="B26">
+        <v>15</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1298,6 +1628,9 @@
           <t>24041 CA SUI / ETT</t>
         </is>
       </c>
+      <c r="B27">
+        <v>15</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1305,6 +1638,9 @@
           <t>2405 Accured Payroll Taxes</t>
         </is>
       </c>
+      <c r="B28">
+        <v>15</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1312,6 +1648,9 @@
           <t>24051 Federal Taxes (941/944)</t>
         </is>
       </c>
+      <c r="B29">
+        <v>15</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1319,6 +1658,9 @@
           <t>24061 Federal Unemployment (940)</t>
         </is>
       </c>
+      <c r="B30">
+        <v>15</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1326,6 +1668,9 @@
           <t>3-65550 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B31">
+        <v>15</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1333,6 +1678,9 @@
           <t>3103 Federal Taxes</t>
         </is>
       </c>
+      <c r="B32">
+        <v>15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1340,6 +1688,9 @@
           <t>4-65550 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B33">
+        <v>15</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1347,6 +1698,9 @@
           <t>5002 Direct Labor - Taxes</t>
         </is>
       </c>
+      <c r="B34">
+        <v>15</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1354,6 +1708,9 @@
           <t>5002 Direct Payroll Taxes</t>
         </is>
       </c>
+      <c r="B35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1361,6 +1718,9 @@
           <t>5005 Direct Support Payroll Taxes</t>
         </is>
       </c>
+      <c r="B36">
+        <v>15</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1368,6 +1728,9 @@
           <t>5102 Direct Labor PR - Taxes</t>
         </is>
       </c>
+      <c r="B37">
+        <v>15</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1375,6 +1738,9 @@
           <t>5102 Direct Payroll Taxes</t>
         </is>
       </c>
+      <c r="B38">
+        <v>15</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1382,6 +1748,9 @@
           <t>51120-000 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B39">
+        <v>15</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1389,6 +1758,9 @@
           <t>5120 Direct Labor - Taxes</t>
         </is>
       </c>
+      <c r="B40">
+        <v>15</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1396,6 +1768,9 @@
           <t>52103-000 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B41">
+        <v>15</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1403,6 +1778,9 @@
           <t>53103-000 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B42">
+        <v>15</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1410,6 +1788,9 @@
           <t>5320 Payroll Taxes - Direct</t>
         </is>
       </c>
+      <c r="B43">
+        <v>15</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1417,6 +1798,9 @@
           <t>60003 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B44">
+        <v>15</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1424,6 +1808,9 @@
           <t>60005 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B45">
+        <v>15</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1431,6 +1818,9 @@
           <t>60014-000 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B46">
+        <v>15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1438,6 +1828,9 @@
           <t>6002 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B47">
+        <v>15</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1445,6 +1838,9 @@
           <t>60020 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B48">
+        <v>15</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1452,6 +1848,9 @@
           <t>60030 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B49">
+        <v>15</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1459,6 +1858,9 @@
           <t>6007 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B50">
+        <v>15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1466,6 +1868,9 @@
           <t>6022 Employee PR - Taxes</t>
         </is>
       </c>
+      <c r="B51">
+        <v>15</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1473,6 +1878,9 @@
           <t>6022 Employee Taxes</t>
         </is>
       </c>
+      <c r="B52">
+        <v>15</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1480,6 +1888,9 @@
           <t>6023 Payroll Tax Expense</t>
         </is>
       </c>
+      <c r="B53">
+        <v>15</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1487,6 +1898,9 @@
           <t>6102 Employee PR - Taxes</t>
         </is>
       </c>
+      <c r="B54">
+        <v>15</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1494,6 +1908,9 @@
           <t>6120 Employee PR - Taxes</t>
         </is>
       </c>
+      <c r="B55">
+        <v>15</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1501,6 +1918,9 @@
           <t>6354 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B56">
+        <v>15</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1508,6 +1928,9 @@
           <t>6402 Employee Taxes</t>
         </is>
       </c>
+      <c r="B57">
+        <v>15</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1515,6 +1938,9 @@
           <t>6452 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B58">
+        <v>15</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1522,6 +1948,9 @@
           <t>65102-000 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B59">
+        <v>15</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1529,12 +1958,18 @@
           <t>6703 Payroll Taxes</t>
         </is>
       </c>
+      <c r="B60">
+        <v>15</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
           <t>62000 Business Licenses and Taxes</t>
         </is>
+      </c>
+      <c r="B61">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1543,15 +1978,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col customWidth="true" max="1" min="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1582,6 +2017,9 @@
           <t>1-65510 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B2">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1589,6 +2027,9 @@
           <t>3-65510 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B3">
+        <v>15</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1596,6 +2037,9 @@
           <t>4-65510 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B4">
+        <v>15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1603,6 +2047,9 @@
           <t>60004 Payroll Processing Fee</t>
         </is>
       </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1610,6 +2057,9 @@
           <t>60005 Payroll Fee</t>
         </is>
       </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1617,6 +2067,9 @@
           <t>60006 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1624,6 +2077,9 @@
           <t>6004 Payroll Fees</t>
         </is>
       </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1631,6 +2087,9 @@
           <t>6006 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B9">
+        <v>15</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1638,6 +2097,9 @@
           <t>60060 Payroll Fees</t>
         </is>
       </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1645,6 +2107,9 @@
           <t>6008 Payroll Fees</t>
         </is>
       </c>
+      <c r="B11">
+        <v>15</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1652,6 +2117,9 @@
           <t>6009 401K Processing Fee</t>
         </is>
       </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1659,6 +2127,9 @@
           <t>6025 Payroll Fees</t>
         </is>
       </c>
+      <c r="B13">
+        <v>15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1666,6 +2137,9 @@
           <t>6030 Payroll Fees</t>
         </is>
       </c>
+      <c r="B14">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1673,6 +2147,9 @@
           <t>6030 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B15">
+        <v>15</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1680,6 +2157,9 @@
           <t>6031 401K Processing Fee</t>
         </is>
       </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1687,6 +2167,9 @@
           <t>6032 Payroll Fees - HSA</t>
         </is>
       </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1694,6 +2177,9 @@
           <t>6110 Payroll Fees</t>
         </is>
       </c>
+      <c r="B18">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1701,6 +2187,9 @@
           <t>6200 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1708,6 +2197,9 @@
           <t>6355 Payroll Fees</t>
         </is>
       </c>
+      <c r="B20">
+        <v>15</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1715,6 +2207,9 @@
           <t>6403 Payroll Fees</t>
         </is>
       </c>
+      <c r="B21">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1722,6 +2217,9 @@
           <t>6407 ADP Payroll Fees</t>
         </is>
       </c>
+      <c r="B22">
+        <v>15</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1729,6 +2227,9 @@
           <t>6453 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B23">
+        <v>15</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1736,6 +2237,9 @@
           <t>65108-000 Payroll Processing Fees</t>
         </is>
       </c>
+      <c r="B24">
+        <v>15</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1743,12 +2247,18 @@
           <t>6558 Payroll Processing Fee</t>
         </is>
       </c>
+      <c r="B25">
+        <v>15</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
           <t>6708 Payroll Processing Fees</t>
         </is>
+      </c>
+      <c r="B26">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1757,15 +2267,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col customWidth="true" max="1" min="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1796,6 +2306,9 @@
           <t>1-14040 Software</t>
         </is>
       </c>
+      <c r="B2">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1803,6 +2316,9 @@
           <t>1-61000 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B3">
+        <v>15</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1810,6 +2326,9 @@
           <t>12700-000 Software Development Costs</t>
         </is>
       </c>
+      <c r="B4">
+        <v>15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1817,6 +2336,9 @@
           <t>13005 Software</t>
         </is>
       </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1824,6 +2346,9 @@
           <t>1301 Computer Software</t>
         </is>
       </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1831,6 +2356,9 @@
           <t>13020 Computer &amp; Software</t>
         </is>
       </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1838,6 +2366,9 @@
           <t>1311 Software - Fixed asset</t>
         </is>
       </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1845,6 +2376,9 @@
           <t>1320 Computers &amp; Software</t>
         </is>
       </c>
+      <c r="B9">
+        <v>15</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1852,6 +2386,9 @@
           <t>1401 Computer Software</t>
         </is>
       </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1859,6 +2396,9 @@
           <t>1501 Software Development</t>
         </is>
       </c>
+      <c r="B11">
+        <v>15</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1866,6 +2406,9 @@
           <t>2-61000 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1873,6 +2416,9 @@
           <t>3-61000 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B13">
+        <v>15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1880,6 +2426,9 @@
           <t>4-64600 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B14">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1887,6 +2436,9 @@
           <t>40000 Membership Dues</t>
         </is>
       </c>
+      <c r="B15">
+        <v>15</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1894,6 +2446,9 @@
           <t>40100-000 Membership Dues</t>
         </is>
       </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1901,6 +2456,9 @@
           <t>40100-008 Community Subscription</t>
         </is>
       </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1908,6 +2466,9 @@
           <t>50020 Software and Tools Subsc...</t>
         </is>
       </c>
+      <c r="B18">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1915,6 +2476,9 @@
           <t>5003 Software &amp; Apps - COGS</t>
         </is>
       </c>
+      <c r="B19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1922,6 +2486,9 @@
           <t>5004 SaaS Software</t>
         </is>
       </c>
+      <c r="B20">
+        <v>15</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1929,6 +2496,9 @@
           <t>5004 Software &amp; App COGS</t>
         </is>
       </c>
+      <c r="B21">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1936,6 +2506,9 @@
           <t>5005 Software &amp; App COGS</t>
         </is>
       </c>
+      <c r="B22">
+        <v>15</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1943,6 +2516,9 @@
           <t>5040 Software COGS - Apps &amp; Other</t>
         </is>
       </c>
+      <c r="B23">
+        <v>15</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1950,6 +2526,9 @@
           <t>5200 Production Software</t>
         </is>
       </c>
+      <c r="B24">
+        <v>15</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1957,6 +2536,9 @@
           <t>5210 Software &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B25">
+        <v>15</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1964,6 +2546,9 @@
           <t>6004 Office Supplies &amp; Software</t>
         </is>
       </c>
+      <c r="B26">
+        <v>15</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1971,6 +2556,9 @@
           <t>60101-000 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B27">
+        <v>15</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1978,6 +2566,9 @@
           <t>6040 Dues &amp; Membership</t>
         </is>
       </c>
+      <c r="B28">
+        <v>15</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1985,6 +2576,9 @@
           <t>6041 Douglas Elliman Dues</t>
         </is>
       </c>
+      <c r="B29">
+        <v>15</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1992,6 +2586,9 @@
           <t>6045 Other Dues &amp; Memberships</t>
         </is>
       </c>
+      <c r="B30">
+        <v>15</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1999,6 +2596,9 @@
           <t>60500 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B31">
+        <v>15</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2006,6 +2606,9 @@
           <t>6052 Association Dues</t>
         </is>
       </c>
+      <c r="B32">
+        <v>15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2013,6 +2616,9 @@
           <t>6055 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B33">
+        <v>15</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2020,6 +2626,9 @@
           <t>6063 Software Expenses</t>
         </is>
       </c>
+      <c r="B34">
+        <v>15</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2027,6 +2636,9 @@
           <t>6100 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2034,6 +2646,9 @@
           <t>6101 Computer Software</t>
         </is>
       </c>
+      <c r="B36">
+        <v>15</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2041,6 +2656,9 @@
           <t>6101 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B37">
+        <v>15</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2048,6 +2666,9 @@
           <t>6130 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B38">
+        <v>15</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2055,6 +2676,9 @@
           <t>6151 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B39">
+        <v>15</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2062,6 +2686,9 @@
           <t>6152 Software &amp; Applications</t>
         </is>
       </c>
+      <c r="B40">
+        <v>15</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2069,6 +2696,9 @@
           <t>6153 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B41">
+        <v>15</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2076,6 +2706,9 @@
           <t>6155 Office Software</t>
         </is>
       </c>
+      <c r="B42">
+        <v>15</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2083,6 +2716,9 @@
           <t>6155 Software &amp; Apps</t>
         </is>
       </c>
+      <c r="B43">
+        <v>15</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2090,6 +2726,9 @@
           <t>61550 Software &amp; Apps</t>
         </is>
       </c>
+      <c r="B44">
+        <v>15</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2097,6 +2736,9 @@
           <t>6158 Software &amp; Apps</t>
         </is>
       </c>
+      <c r="B45">
+        <v>15</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2104,6 +2746,9 @@
           <t>6158 Software &amp; apps</t>
         </is>
       </c>
+      <c r="B46">
+        <v>15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2111,6 +2756,9 @@
           <t>6200 Computer Software &amp; Inter...</t>
         </is>
       </c>
+      <c r="B47">
+        <v>15</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2118,6 +2766,9 @@
           <t>6200 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B48">
+        <v>15</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2125,6 +2776,9 @@
           <t>6201 Dues &amp; Subscription</t>
         </is>
       </c>
+      <c r="B49">
+        <v>15</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2132,6 +2786,9 @@
           <t>6203 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B50">
+        <v>15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2139,6 +2796,9 @@
           <t>6204 Software Subscriptions</t>
         </is>
       </c>
+      <c r="B51">
+        <v>15</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2146,6 +2806,9 @@
           <t>6205 Software &amp; Computer Expen...</t>
         </is>
       </c>
+      <c r="B52">
+        <v>15</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2153,6 +2816,9 @@
           <t>6206 Software &amp; Apps</t>
         </is>
       </c>
+      <c r="B53">
+        <v>15</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2160,6 +2826,9 @@
           <t>6215 Computer Software</t>
         </is>
       </c>
+      <c r="B54">
+        <v>15</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2167,6 +2836,9 @@
           <t>62275 Dues &amp; Subscription</t>
         </is>
       </c>
+      <c r="B55">
+        <v>15</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2174,6 +2846,9 @@
           <t>6250 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B56">
+        <v>15</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2181,6 +2856,9 @@
           <t>62500 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B57">
+        <v>15</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2188,6 +2866,9 @@
           <t>62500 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B58">
+        <v>15</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2195,6 +2876,9 @@
           <t>62500 Office Supplies &amp; Software</t>
         </is>
       </c>
+      <c r="B59">
+        <v>15</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2202,6 +2886,9 @@
           <t>6255 Subscriptions</t>
         </is>
       </c>
+      <c r="B60">
+        <v>15</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2209,6 +2896,9 @@
           <t>6275 Software, Apps, Subscriptions</t>
         </is>
       </c>
+      <c r="B61">
+        <v>15</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2216,6 +2906,9 @@
           <t>6300 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B62">
+        <v>15</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2223,6 +2916,9 @@
           <t>6300 Memberships &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B63">
+        <v>15</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2230,6 +2926,9 @@
           <t>6300 Systems &amp; Software</t>
         </is>
       </c>
+      <c r="B64">
+        <v>15</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2237,6 +2936,9 @@
           <t>6301 Software &amp; Applications</t>
         </is>
       </c>
+      <c r="B65">
+        <v>15</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2244,6 +2946,9 @@
           <t>6302 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B66">
+        <v>15</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2251,6 +2956,9 @@
           <t>63031 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B67">
+        <v>15</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2258,6 +2966,9 @@
           <t>6307 Software &amp; Apps</t>
         </is>
       </c>
+      <c r="B68">
+        <v>15</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2265,6 +2976,9 @@
           <t>6352 Apps &amp; Software</t>
         </is>
       </c>
+      <c r="B69">
+        <v>15</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2272,6 +2986,9 @@
           <t>6353 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B70">
+        <v>15</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2279,6 +2996,9 @@
           <t>6401 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B71">
+        <v>15</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2286,6 +3006,9 @@
           <t>6404 Software Expenses</t>
         </is>
       </c>
+      <c r="B72">
+        <v>15</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2293,6 +3016,9 @@
           <t>6405 Software</t>
         </is>
       </c>
+      <c r="B73">
+        <v>15</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2300,6 +3026,9 @@
           <t>6450 Office Supplies &amp; Software</t>
         </is>
       </c>
+      <c r="B74">
+        <v>15</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2307,6 +3036,9 @@
           <t>65270-000 Dues and Subscriptions</t>
         </is>
       </c>
+      <c r="B75">
+        <v>15</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2314,6 +3046,9 @@
           <t>6600 Office Supplies &amp; Software</t>
         </is>
       </c>
+      <c r="B76">
+        <v>15</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2321,6 +3056,9 @@
           <t>6715 Software Expense</t>
         </is>
       </c>
+      <c r="B77">
+        <v>15</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2328,6 +3066,9 @@
           <t>6903 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B78">
+        <v>15</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2335,12 +3076,18 @@
           <t>69030 Dues &amp; Subscriptions</t>
         </is>
       </c>
+      <c r="B79">
+        <v>15</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
           <t>69030 Dues and Subscriptions</t>
         </is>
+      </c>
+      <c r="B80">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2349,15 +3096,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col customWidth="true" max="1" min="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2388,6 +3135,9 @@
           <t>1-67000 Telephone Expense</t>
         </is>
       </c>
+      <c r="B2">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2395,6 +3145,9 @@
           <t>1-67700 Utilities</t>
         </is>
       </c>
+      <c r="B3">
+        <v>15</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2402,6 +3155,9 @@
           <t>1303 Phone Hardware</t>
         </is>
       </c>
+      <c r="B4">
+        <v>15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2409,6 +3165,9 @@
           <t>3-61750 Computer and Internet Expenses</t>
         </is>
       </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2416,6 +3175,9 @@
           <t>3-67000 Telephone Expense</t>
         </is>
       </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2423,6 +3185,9 @@
           <t>3-67700 Utilities</t>
         </is>
       </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2430,6 +3195,9 @@
           <t>4-67000 Telephone Expense</t>
         </is>
       </c>
+      <c r="B8">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2437,6 +3205,9 @@
           <t>4-67700 Utilities</t>
         </is>
       </c>
+      <c r="B9">
+        <v>15</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2444,6 +3215,9 @@
           <t>5511 Cell Phone Expense - Sales</t>
         </is>
       </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2451,6 +3225,9 @@
           <t>6045 Computer and Internet Expen...</t>
         </is>
       </c>
+      <c r="B11">
+        <v>15</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2458,6 +3235,9 @@
           <t>6062 Utilities</t>
         </is>
       </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2465,6 +3245,9 @@
           <t>6063 Telephone</t>
         </is>
       </c>
+      <c r="B13">
+        <v>15</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2472,6 +3255,9 @@
           <t>6064 Internet Expense</t>
         </is>
       </c>
+      <c r="B14">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2479,6 +3265,9 @@
           <t>6065 Utilities</t>
         </is>
       </c>
+      <c r="B15">
+        <v>15</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2486,6 +3275,9 @@
           <t>6100 Computer and Internet</t>
         </is>
       </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2493,6 +3285,9 @@
           <t>6101 Gas</t>
         </is>
       </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2500,6 +3295,9 @@
           <t>6103 Phone service</t>
         </is>
       </c>
+      <c r="B18">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2507,6 +3305,9 @@
           <t>6115 Utilities</t>
         </is>
       </c>
+      <c r="B19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2514,6 +3315,9 @@
           <t>6117 Internet &amp; Telephone</t>
         </is>
       </c>
+      <c r="B20">
+        <v>15</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2521,6 +3325,9 @@
           <t>6154 Electric &amp; Gas</t>
         </is>
       </c>
+      <c r="B21">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2528,6 +3335,9 @@
           <t>6155 Phone &amp; Internet Expenses</t>
         </is>
       </c>
+      <c r="B22">
+        <v>15</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2535,6 +3345,9 @@
           <t>61600 Utilities</t>
         </is>
       </c>
+      <c r="B23">
+        <v>15</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2542,6 +3355,9 @@
           <t>61700 Computer and Internet Expe...</t>
         </is>
       </c>
+      <c r="B24">
+        <v>15</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2549,6 +3365,9 @@
           <t>61700 Telephone Expense</t>
         </is>
       </c>
+      <c r="B25">
+        <v>15</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2556,6 +3375,9 @@
           <t>6200 Computer and Internet Expenses</t>
         </is>
       </c>
+      <c r="B26">
+        <v>15</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2563,6 +3385,9 @@
           <t>62000 Office &amp; Utility Expenses</t>
         </is>
       </c>
+      <c r="B27">
+        <v>15</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2570,6 +3395,9 @@
           <t>6203 Phone/Internet</t>
         </is>
       </c>
+      <c r="B28">
+        <v>15</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2577,6 +3405,9 @@
           <t>62030 Gas/Mileage</t>
         </is>
       </c>
+      <c r="B29">
+        <v>15</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2584,6 +3415,9 @@
           <t>6204 Internet &amp; Telephone Expe...</t>
         </is>
       </c>
+      <c r="B30">
+        <v>15</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2591,6 +3425,9 @@
           <t>62051 Utilities</t>
         </is>
       </c>
+      <c r="B31">
+        <v>15</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2598,6 +3435,9 @@
           <t>6207 Vehicle Gas &amp; Fuel</t>
         </is>
       </c>
+      <c r="B32">
+        <v>15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2605,6 +3445,9 @@
           <t>6225 Utilities</t>
         </is>
       </c>
+      <c r="B33">
+        <v>15</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2612,6 +3455,9 @@
           <t>6230 Cell Phone</t>
         </is>
       </c>
+      <c r="B34">
+        <v>15</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2619,6 +3465,9 @@
           <t>6231 Internet</t>
         </is>
       </c>
+      <c r="B35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2626,6 +3475,9 @@
           <t>6233 Phone Service</t>
         </is>
       </c>
+      <c r="B36">
+        <v>15</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2633,6 +3485,9 @@
           <t>6256 Telephone &amp; Internet</t>
         </is>
       </c>
+      <c r="B37">
+        <v>15</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2640,6 +3495,9 @@
           <t>6257 Utilities</t>
         </is>
       </c>
+      <c r="B38">
+        <v>15</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2647,6 +3505,9 @@
           <t>62850 Utilities</t>
         </is>
       </c>
+      <c r="B39">
+        <v>15</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2654,6 +3515,9 @@
           <t>6301 Gas</t>
         </is>
       </c>
+      <c r="B40">
+        <v>15</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2661,6 +3525,9 @@
           <t>63020 Gas / Electric Charging</t>
         </is>
       </c>
+      <c r="B41">
+        <v>15</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2668,6 +3535,9 @@
           <t>6308 Telephone &amp; Internet</t>
         </is>
       </c>
+      <c r="B42">
+        <v>15</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2675,6 +3545,9 @@
           <t>6366 Telephone</t>
         </is>
       </c>
+      <c r="B43">
+        <v>15</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2682,6 +3555,9 @@
           <t>6367 Utilities</t>
         </is>
       </c>
+      <c r="B44">
+        <v>15</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2689,6 +3565,9 @@
           <t>6375 Utilities</t>
         </is>
       </c>
+      <c r="B45">
+        <v>15</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2696,6 +3575,9 @@
           <t>64020 Utilities</t>
         </is>
       </c>
+      <c r="B46">
+        <v>15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2703,6 +3585,9 @@
           <t>6403 Internet</t>
         </is>
       </c>
+      <c r="B47">
+        <v>15</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2710,6 +3595,9 @@
           <t>64030 Telephone</t>
         </is>
       </c>
+      <c r="B48">
+        <v>15</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2717,6 +3605,9 @@
           <t>6404 Telephone</t>
         </is>
       </c>
+      <c r="B49">
+        <v>15</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2724,6 +3615,9 @@
           <t>64040 Internet</t>
         </is>
       </c>
+      <c r="B50">
+        <v>15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2731,6 +3625,9 @@
           <t>65240-001 Telephone Expense</t>
         </is>
       </c>
+      <c r="B51">
+        <v>15</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2738,6 +3635,9 @@
           <t>6653 Electricity</t>
         </is>
       </c>
+      <c r="B52">
+        <v>15</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2745,6 +3645,9 @@
           <t>6654 Internet &amp; TV Services</t>
         </is>
       </c>
+      <c r="B53">
+        <v>15</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2752,6 +3655,9 @@
           <t>6655 Other Utilities</t>
         </is>
       </c>
+      <c r="B54">
+        <v>15</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2759,6 +3665,9 @@
           <t>6750 Telephone Expense</t>
         </is>
       </c>
+      <c r="B55">
+        <v>15</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2766,6 +3675,9 @@
           <t>6800 Telephone Expense</t>
         </is>
       </c>
+      <c r="B56">
+        <v>15</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2773,6 +3685,9 @@
           <t>6800 Utilities</t>
         </is>
       </c>
+      <c r="B57">
+        <v>15</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2780,6 +3695,9 @@
           <t>6801 Cable &amp; Internet</t>
         </is>
       </c>
+      <c r="B58">
+        <v>15</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2787,6 +3705,9 @@
           <t>6801 Gas &amp; Car Charge</t>
         </is>
       </c>
+      <c r="B59">
+        <v>15</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2794,6 +3715,9 @@
           <t>6801 Gas &amp; Fuel</t>
         </is>
       </c>
+      <c r="B60">
+        <v>15</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2801,6 +3725,9 @@
           <t>6806 Telephone</t>
         </is>
       </c>
+      <c r="B61">
+        <v>15</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2808,6 +3735,9 @@
           <t>68100 Telephone Expense</t>
         </is>
       </c>
+      <c r="B62">
+        <v>15</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2815,6 +3745,9 @@
           <t>6850 Telephone</t>
         </is>
       </c>
+      <c r="B63">
+        <v>15</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2822,6 +3755,9 @@
           <t>68600 Utilities</t>
         </is>
       </c>
+      <c r="B64">
+        <v>15</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2829,12 +3765,18 @@
           <t>6900 Utilities</t>
         </is>
       </c>
+      <c r="B65">
+        <v>15</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
           <t>6950 Utilities</t>
         </is>
+      </c>
+      <c r="B66">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>